<commit_message>
Update pending-points status (July 2569): 21 points from BMA traffic report
- Add data/sheets/13_Pending_Update.json (21 points, 8 status groups)
- Tag 26 rows with status_latest/status_group in combined data, sheet 08, geojson
- Set progress to 100% for 5 completed points (6 rows)
- Add 'Latest Pending-Points Update' section to Status tab in dashboard
- Update README with July 2569 data update summary
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Spatial Lineage" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Corridors" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_New &amp; Dropout" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Pending Update" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9005,6 +9006,1045 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>อัปเดตสถานะจุดฝืด — รายงานจุดฝืดที่ยังไม่ได้ดำเนินการ (สจส. ก.ค. 2569)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ลำดับ</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ปี</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ชื่อจุด</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>เขต</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>โซน</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ผู้รับผิดชอบ</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>สถานะล่าสุด</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>กลุ่มสถานะ</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>lon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2567</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>คอขวดปากทางลาดพร้าว (ช่วงโค้งถนนลาดพร้าวก่อนตัดกับถนนพหลโยธิน)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>จตุจักร</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>กรุงเทพเหนือ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>สน.วิภาวดีไม่ให้เปิดใช้งานสัญญาณไฟด้านถนนลาดพร้าว</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ติดข้อจำกัดหน่วยงานอื่น</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>13.81327778</v>
+      </c>
+      <c r="J4" t="n">
+        <v>100.5603611</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2567</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>แยกต่างระดับราชพฤกษ์ - รัชดาภิเษก</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ธนบุรี</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>กรุงธนเหนือ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>กรมทางหลวงชนบท</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>อยู่ในความรับผิดชอบ ทช.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>นอกอำนาจ กทม.</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>13.7154111</v>
+      </c>
+      <c r="J5" t="n">
+        <v>100.4782633</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2567</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>คอขวดถนนหัวหมาก (ซอยรามคำแหง24) ช่วงตั้งแต่แยกกวนอา-ม.เอแบค</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>บางกะปิ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>กรุงเทพตะวันออก</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>สนย.ดำเนินการขยายถนนแล้วเสร็จ</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>13.755223</v>
+      </c>
+      <c r="J6" t="n">
+        <v>100.626843</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2567</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>จุดกลับรถหน้าไปรษณีย์ย่อยบางบอน ถนนเอกชัย</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>บางบอน</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>กรุงธนใต้</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ปาดบาทวิถีให้กลับรถได้ 2 เลนเรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>13.661834</v>
+      </c>
+      <c r="J7" t="n">
+        <v>100.403637</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>แยกพลาธิการทหารอากาศ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ดอนเมือง</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>กรุงเทพเหนือ</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ติดตั้งสัญญาณไฟ adaptive แล้ว</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>13.90183333</v>
+      </c>
+      <c r="J8" t="n">
+        <v>100.6122222</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>คอขวดถนนสามเสนช่วงก่อนถึงแยกซังฮี้ ทางทิศใต้</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ดุสิต</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง สน.สามเสนจัดการจราจร</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>13.77983333</v>
+      </c>
+      <c r="J9" t="n">
+        <v>100.5091389</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2567/2568</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>แยกซังฮี้</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ดุสิต</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>13.778386</v>
+      </c>
+      <c r="J10" t="n">
+        <v>100.508418</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2567/2568</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>คอขวดโรงเรียนซางตาครู้สคอนแวนต์ ถนนเทศบาลสาย 1 (ซอยอรุณอมรินทร์ 4)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ธนบุรี</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>กรุงธนเหนือ</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>มาตรการชั่วคราว</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>13.737245</v>
+      </c>
+      <c r="J11" t="n">
+        <v>100.49404</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>คอขวดทางขึ้นสะพานวัชรพล ถนนประดิษฐ์มนูธรรม</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>บางเขน</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>กรุงเทพเหนือ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>มาตรการชั่วคราว</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>13.85005556</v>
+      </c>
+      <c r="J12" t="n">
+        <v>100.6393611</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2567/2568</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>แยกถนนเพชรเกษม-พุทธมณฑลสาย 1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ภาษีเจริญ</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>กรุงธนใต้</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ขยับจุดกลับรถ 50 ม. + ย้ายทางข้าม เรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>13.712633</v>
+      </c>
+      <c r="J13" t="n">
+        <v>100.428358</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>จุดกลับรถใกล้แยกพญาไท</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ราชเทวี</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ความสูงช่องลอดกลับรถไม่เพียงพอ</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>13.75775</v>
+      </c>
+      <c r="J14" t="n">
+        <v>100.5349167</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>แยกกำแพงเพชร 7-อโศกดินแดง</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ราชเทวี</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ยังไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ปี 69 ได้งบ adaptive อยู่ระหว่างอนุมัติจ้าง</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>รองบปี 2569</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>13.74999</v>
+      </c>
+      <c r="J15" t="n">
+        <v>100.563632</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>แยกมักกะสัน (แยกหมอเหล็ง)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ราชเทวี</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ยังไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีส้ม</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>13.754902</v>
+      </c>
+      <c r="J16" t="n">
+        <v>100.54214</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>บริเวณทางเชื่อมระหว่างมอเตอร์เวย์กับถนนพระราม 9</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>สวนหลวง</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>กรุงเทพใต้</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>กทพ.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>อยู่ในความรับผิดชอบ กทพ.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>นอกอำนาจ กทม.</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>13.742533</v>
+      </c>
+      <c r="J17" t="n">
+        <v>100.63775</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>จุดกลับรถหน้าหมู่บ้านศรีประจักษ์ ถนนรามคำแหง</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>สะพานสูง</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>กรุงเทพตะวันออก</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>13.787472</v>
+      </c>
+      <c r="J18" t="n">
+        <v>100.6927</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>จุดกลับรถหน้าหมู่บ้านสัมมากร ประตู 2 ถนนรามคำแหง</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>สะพานสูง</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>กรุงเทพตะวันออก</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>13.777225</v>
+      </c>
+      <c r="J19" t="n">
+        <v>100.674031</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>แยก คปอ.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>สายไหม</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>กรุงเทพเหนือ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ติดตั้งสัญญาณไฟ adaptive แล้ว</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>13.92358333</v>
+      </c>
+      <c r="J20" t="n">
+        <v>100.625</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>จุดกลับรถหน้าโรงพยาบาลเวชการุณย์รัศมิ์</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>หนองจอก</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>กรุงเทพตะวันออก</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ยังไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ความกว้างถนนไม่พอปรับ 2→4 ช่อง</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>13.85579832</v>
+      </c>
+      <c r="J21" t="n">
+        <v>100.8527928</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>จุดกลับรถหน้าโตโยต้าภูมิพัฒนา</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>หนองจอก</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>กรุงเทพตะวันออก</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ยังไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ความกว้างถนนไม่พอปรับ 2→4 ช่อง</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>13.85579832</v>
+      </c>
+      <c r="J22" t="n">
+        <v>100.8527928</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2567/2568</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>คอขวดทางขึ้นสะพานข้ามคลองแสนแสบ ด้านถนนเพชรบุรี</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ห้วยขวาง</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>สนย.ดำเนินการปรับปรุงสะพาน (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>กำลังดำเนินการ</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>13.74208333</v>
+      </c>
+      <c r="J23" t="n">
+        <v>100.59625</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2568</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>แยกจุดใต้ทางด่วนพระราม 9 (หน้าโรงพยาบาลปิยะเวท)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ห้วยขวาง</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>กรุงเทพกลาง</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ยังไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ปี 69 ได้งบ adaptive อยู่ระหว่างอนุมัติจ้าง</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>รองบปี 2569</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>13.7543877</v>
+      </c>
+      <c r="J24" t="n">
+        <v>100.5796209</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14047,7 +15087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T473"/>
+  <dimension ref="A1:V473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14180,6 +15220,16 @@
           <t>longitude</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>status_latest</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>status_group</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -32119,6 +33169,16 @@
       <c r="T276" s="9" t="n">
         <v>100.4782633</v>
       </c>
+      <c r="U276" t="inlineStr">
+        <is>
+          <t>อยู่ในความรับผิดชอบ ทช.</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>นอกอำนาจ กทม.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="9" t="n">
@@ -34934,6 +35994,16 @@
       <c r="T315" s="9" t="n">
         <v>100.5603611</v>
       </c>
+      <c r="U315" t="inlineStr">
+        <is>
+          <t>สน.วิภาวดีไม่ให้เปิดใช้งานสัญญาณไฟด้านถนนลาดพร้าว</t>
+        </is>
+      </c>
+      <c r="V315" t="inlineStr">
+        <is>
+          <t>ติดข้อจำกัดหน่วยงานอื่น</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="9" t="n">
@@ -35656,6 +36726,16 @@
       <c r="T325" s="9" t="n">
         <v>100.5091389</v>
       </c>
+      <c r="U325" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง</t>
+        </is>
+      </c>
+      <c r="V325" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="9" t="n">
@@ -35729,6 +36809,16 @@
       <c r="T326" s="9" t="n">
         <v>100.508418</v>
       </c>
+      <c r="U326" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง</t>
+        </is>
+      </c>
+      <c r="V326" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="9" t="n">
@@ -36019,6 +37109,16 @@
       <c r="T330" s="9" t="n">
         <v>100.49404</v>
       </c>
+      <c r="U330" t="inlineStr">
+        <is>
+          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="V330" t="inlineStr">
+        <is>
+          <t>มาตรการชั่วคราว</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="9" t="n">
@@ -36570,7 +37670,7 @@
         </is>
       </c>
       <c r="L338" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M338" s="9" t="n">
         <v>0</v>
@@ -36595,6 +37695,16 @@
       </c>
       <c r="T338" s="9" t="n">
         <v>100.626843</v>
+      </c>
+      <c r="U338" t="inlineStr">
+        <is>
+          <t>สนย.ดำเนินการขยายถนนแล้วเสร็จ</t>
+        </is>
+      </c>
+      <c r="V338" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="339">
@@ -37653,7 +38763,7 @@
         </is>
       </c>
       <c r="L353" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M353" s="9" t="n">
         <v>0</v>
@@ -37678,6 +38788,16 @@
       </c>
       <c r="T353" s="9" t="n">
         <v>100.403637</v>
+      </c>
+      <c r="U353" t="inlineStr">
+        <is>
+          <t>ปาดบาทวิถีให้กลับรถได้ 2 เลนเรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="V353" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="354">
@@ -38664,7 +39784,7 @@
         </is>
       </c>
       <c r="L367" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M367" s="9" t="n">
         <v>0</v>
@@ -38689,6 +39809,16 @@
       </c>
       <c r="T367" s="9" t="n">
         <v>100.428358</v>
+      </c>
+      <c r="U367" t="inlineStr">
+        <is>
+          <t>ขยับจุดกลับรถ 50 ม. + ย้ายทางข้าม เรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="V367" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="368">
@@ -40782,6 +41912,16 @@
       </c>
       <c r="T396" s="9" t="n">
         <v>100.59625</v>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>สนย.ดำเนินการปรับปรุงสะพาน (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>กำลังดำเนินการ</t>
+        </is>
       </c>
     </row>
     <row r="397">
@@ -44515,6 +45655,16 @@
       <c r="T452" s="9" t="n">
         <v>100.63775</v>
       </c>
+      <c r="U452" t="inlineStr">
+        <is>
+          <t>อยู่ในความรับผิดชอบ กทพ.</t>
+        </is>
+      </c>
+      <c r="V452" t="inlineStr">
+        <is>
+          <t>นอกอำนาจ กทม.</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="9" t="n">
@@ -44583,6 +45733,16 @@
       <c r="T453" s="9" t="n">
         <v>100.49404</v>
       </c>
+      <c r="U453" t="inlineStr">
+        <is>
+          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="V453" t="inlineStr">
+        <is>
+          <t>มาตรการชั่วคราว</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="9" t="n">
@@ -44651,6 +45811,16 @@
       <c r="T454" s="9" t="n">
         <v>100.5091389</v>
       </c>
+      <c r="U454" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง สน.สามเสนจัดการจราจร</t>
+        </is>
+      </c>
+      <c r="V454" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="9" t="n">
@@ -44720,6 +45890,16 @@
       <c r="T455" s="9" t="n">
         <v>100.508418</v>
       </c>
+      <c r="U455" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีม่วง สน.สามเสนจัดการจราจร</t>
+        </is>
+      </c>
+      <c r="V455" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="9" t="n">
@@ -44787,6 +45967,16 @@
       </c>
       <c r="T456" s="9" t="n">
         <v>100.5349167</v>
+      </c>
+      <c r="U456" t="inlineStr">
+        <is>
+          <t>ความสูงช่องลอดกลับรถไม่เพียงพอ</t>
+        </is>
+      </c>
+      <c r="V456" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
       </c>
     </row>
     <row r="457">
@@ -44852,6 +46042,16 @@
       <c r="T457" s="9" t="n">
         <v>100.563632</v>
       </c>
+      <c r="U457" t="inlineStr">
+        <is>
+          <t>ปี 69 ได้งบ adaptive อยู่ระหว่างอนุมัติจ้าง</t>
+        </is>
+      </c>
+      <c r="V457" t="inlineStr">
+        <is>
+          <t>รองบปี 2569</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="9" t="n">
@@ -44916,6 +46116,16 @@
       <c r="T458" s="9" t="n">
         <v>100.54214</v>
       </c>
+      <c r="U458" t="inlineStr">
+        <is>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้าสายสีส้ม</t>
+        </is>
+      </c>
+      <c r="V458" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="9" t="n">
@@ -44983,6 +46193,16 @@
       </c>
       <c r="T459" s="9" t="n">
         <v>100.6393611</v>
+      </c>
+      <c r="U459" t="inlineStr">
+        <is>
+          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว</t>
+        </is>
+      </c>
+      <c r="V459" t="inlineStr">
+        <is>
+          <t>มาตรการชั่วคราว</t>
+        </is>
       </c>
     </row>
     <row r="460">
@@ -45116,6 +46336,16 @@
       <c r="T461" s="9" t="n">
         <v>100.59625</v>
       </c>
+      <c r="U461" t="inlineStr">
+        <is>
+          <t>สนย.ดำเนินการปรับปรุงสะพาน (ซ้ำปี 68)</t>
+        </is>
+      </c>
+      <c r="V461" t="inlineStr">
+        <is>
+          <t>กำลังดำเนินการ</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="9" t="n">
@@ -45180,6 +46410,16 @@
       <c r="T462" s="9" t="n">
         <v>100.5796209</v>
       </c>
+      <c r="U462" t="inlineStr">
+        <is>
+          <t>ปี 69 ได้งบ adaptive อยู่ระหว่างอนุมัติจ้าง</t>
+        </is>
+      </c>
+      <c r="V462" t="inlineStr">
+        <is>
+          <t>รองบปี 2569</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="9" t="n">
@@ -45244,6 +46484,16 @@
       <c r="T463" s="9" t="n">
         <v>100.8527928</v>
       </c>
+      <c r="U463" t="inlineStr">
+        <is>
+          <t>ความกว้างถนนไม่พอปรับ 2→4 ช่อง</t>
+        </is>
+      </c>
+      <c r="V463" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" s="9" t="n">
@@ -45308,6 +46558,16 @@
       <c r="T464" s="9" t="n">
         <v>100.8527928</v>
       </c>
+      <c r="U464" t="inlineStr">
+        <is>
+          <t>ความกว้างถนนไม่พอปรับ 2→4 ช่อง</t>
+        </is>
+      </c>
+      <c r="V464" t="inlineStr">
+        <is>
+          <t>ข้อจำกัดกายภาพ</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" s="9" t="n">
@@ -45351,7 +46611,7 @@
       </c>
       <c r="K465" s="9" t="inlineStr"/>
       <c r="L465" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M465" s="9" t="n">
         <v>0</v>
@@ -45376,6 +46636,16 @@
       </c>
       <c r="T465" s="9" t="n">
         <v>100.428358</v>
+      </c>
+      <c r="U465" t="inlineStr">
+        <is>
+          <t>ขยับจุดกลับรถ 50 ม. + ย้ายทางข้าม เรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="V465" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="466">
@@ -45445,6 +46715,16 @@
       <c r="T466" s="9" t="n">
         <v>100.6927</v>
       </c>
+      <c r="U466" t="inlineStr">
+        <is>
+          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร</t>
+        </is>
+      </c>
+      <c r="V466" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="9" t="n">
@@ -45513,6 +46793,16 @@
       <c r="T467" s="9" t="n">
         <v>100.674031</v>
       </c>
+      <c r="U467" t="inlineStr">
+        <is>
+          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร</t>
+        </is>
+      </c>
+      <c r="V467" t="inlineStr">
+        <is>
+          <t>ติดก่อสร้างรถไฟฟ้า</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" s="9" t="n">
@@ -45555,7 +46845,7 @@
       </c>
       <c r="K468" s="9" t="inlineStr"/>
       <c r="L468" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M468" s="9" t="n">
         <v>0</v>
@@ -45580,6 +46870,16 @@
       </c>
       <c r="T468" s="9" t="n">
         <v>100.6122222</v>
+      </c>
+      <c r="U468" t="inlineStr">
+        <is>
+          <t>ติดตั้งสัญญาณไฟ adaptive แล้ว</t>
+        </is>
+      </c>
+      <c r="V468" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="469">
@@ -45623,7 +46923,7 @@
       </c>
       <c r="K469" s="9" t="inlineStr"/>
       <c r="L469" s="9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M469" s="9" t="n">
         <v>0</v>
@@ -45648,6 +46948,16 @@
       </c>
       <c r="T469" s="9" t="n">
         <v>100.625</v>
+      </c>
+      <c r="U469" t="inlineStr">
+        <is>
+          <t>ติดตั้งสัญญาณไฟ adaptive แล้ว</t>
+        </is>
+      </c>
+      <c r="V469" t="inlineStr">
+        <is>
+          <t>เสร็จแล้ว</t>
+        </is>
       </c>
     </row>
     <row r="470">

</xml_diff>

<commit_message>
Fix: separate Makkasan railway junction from Mo Leng intersection
- 'แยกมักกะสัน' (FY2567, FY2568) renamed to 'แยกมักกะสัน (สามแยกทางรถไฟ)'
  and moved to correct coordinates (13.7540, 100.5423) ~100m south
- Previously shared identical coordinates with 'แยกมักกะสัน (แยกหมอเหล็ง)'
  (Ratchaprarop x Si Ayutthaya) causing overlapping contradictory markers
- Applied to combined_data.json, sheet 08, geojson, data.xlsx
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -39975,7 +39975,7 @@
       </c>
       <c r="C370" s="9" t="inlineStr">
         <is>
-          <t>แยกมักกะสัน</t>
+          <t>แยกมักกะสัน (สามแยกทางรถไฟ)</t>
         </is>
       </c>
       <c r="D370" s="9" t="inlineStr">
@@ -40032,10 +40032,10 @@
         <v>0</v>
       </c>
       <c r="S370" s="9" t="n">
-        <v>13.754904</v>
+        <v>13.754</v>
       </c>
       <c r="T370" s="9" t="n">
-        <v>100.542131</v>
+        <v>100.5423</v>
       </c>
     </row>
     <row r="371">
@@ -42139,7 +42139,7 @@
       </c>
       <c r="C400" s="9" t="inlineStr">
         <is>
-          <t>แยกมักกะสัน</t>
+          <t>แยกมักกะสัน (สามแยกทางรถไฟ)</t>
         </is>
       </c>
       <c r="D400" s="9" t="inlineStr">
@@ -42192,10 +42192,10 @@
         <v>0</v>
       </c>
       <c r="S400" s="9" t="n">
-        <v>13.754904</v>
+        <v>13.754</v>
       </c>
       <c r="T400" s="9" t="n">
-        <v>100.542131</v>
+        <v>100.5423</v>
       </c>
     </row>
     <row r="401">

</xml_diff>

<commit_message>
Dashboard: FY2568 agency split (BMA / non-BMA / unspecified); fill EXAT as agency for Motorway-Rama 9 link per July 2569 report
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -45626,7 +45626,11 @@
       </c>
       <c r="H452" s="9" t="inlineStr"/>
       <c r="I452" s="9" t="inlineStr"/>
-      <c r="J452" s="9" t="inlineStr"/>
+      <c r="J452" s="9" t="inlineStr">
+        <is>
+          <t>การทางพิเศษแห่งประเทศไทย</t>
+        </is>
+      </c>
       <c r="K452" s="9" t="inlineStr"/>
       <c r="L452" s="9" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Data: assign BMA as responsible agency for 28 unspecified FY2568 points (per user confirmation)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9606,7 +9606,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ยังไม่ระบุ</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -9652,7 +9652,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ยังไม่ระบุ</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ยังไม่ระบุ</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -9928,7 +9928,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>ยังไม่ระบุ</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ยังไม่ระบุ</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -42301,7 +42301,11 @@
       </c>
       <c r="H402" s="9" t="inlineStr"/>
       <c r="I402" s="9" t="inlineStr"/>
-      <c r="J402" s="9" t="inlineStr"/>
+      <c r="J402" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K402" s="9" t="inlineStr"/>
       <c r="L402" s="9" t="n">
         <v>100</v>
@@ -42569,7 +42573,11 @@
       </c>
       <c r="H406" s="9" t="inlineStr"/>
       <c r="I406" s="9" t="inlineStr"/>
-      <c r="J406" s="9" t="inlineStr"/>
+      <c r="J406" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K406" s="9" t="inlineStr"/>
       <c r="L406" s="9" t="n">
         <v>100</v>
@@ -42702,7 +42710,11 @@
       </c>
       <c r="H408" s="9" t="inlineStr"/>
       <c r="I408" s="9" t="inlineStr"/>
-      <c r="J408" s="9" t="inlineStr"/>
+      <c r="J408" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K408" s="9" t="inlineStr"/>
       <c r="L408" s="9" t="n">
         <v>100</v>
@@ -42766,7 +42778,11 @@
       </c>
       <c r="H409" s="9" t="inlineStr"/>
       <c r="I409" s="9" t="inlineStr"/>
-      <c r="J409" s="9" t="inlineStr"/>
+      <c r="J409" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K409" s="9" t="inlineStr"/>
       <c r="L409" s="9" t="n">
         <v>100</v>
@@ -42830,7 +42846,11 @@
       </c>
       <c r="H410" s="9" t="inlineStr"/>
       <c r="I410" s="9" t="inlineStr"/>
-      <c r="J410" s="9" t="inlineStr"/>
+      <c r="J410" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K410" s="9" t="inlineStr"/>
       <c r="L410" s="9" t="n">
         <v>100</v>
@@ -42963,7 +42983,11 @@
       </c>
       <c r="H412" s="9" t="inlineStr"/>
       <c r="I412" s="9" t="inlineStr"/>
-      <c r="J412" s="9" t="inlineStr"/>
+      <c r="J412" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K412" s="9" t="inlineStr"/>
       <c r="L412" s="9" t="n">
         <v>100</v>
@@ -43027,7 +43051,11 @@
       </c>
       <c r="H413" s="9" t="inlineStr"/>
       <c r="I413" s="9" t="inlineStr"/>
-      <c r="J413" s="9" t="inlineStr"/>
+      <c r="J413" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K413" s="9" t="inlineStr"/>
       <c r="L413" s="9" t="n">
         <v>100</v>
@@ -43091,7 +43119,11 @@
       </c>
       <c r="H414" s="9" t="inlineStr"/>
       <c r="I414" s="9" t="inlineStr"/>
-      <c r="J414" s="9" t="inlineStr"/>
+      <c r="J414" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K414" s="9" t="inlineStr"/>
       <c r="L414" s="9" t="n">
         <v>100</v>
@@ -43155,7 +43187,11 @@
       </c>
       <c r="H415" s="9" t="inlineStr"/>
       <c r="I415" s="9" t="inlineStr"/>
-      <c r="J415" s="9" t="inlineStr"/>
+      <c r="J415" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K415" s="9" t="inlineStr"/>
       <c r="L415" s="9" t="n">
         <v>100</v>
@@ -43219,7 +43255,11 @@
       </c>
       <c r="H416" s="9" t="inlineStr"/>
       <c r="I416" s="9" t="inlineStr"/>
-      <c r="J416" s="9" t="inlineStr"/>
+      <c r="J416" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K416" s="9" t="inlineStr"/>
       <c r="L416" s="9" t="n">
         <v>100</v>
@@ -43351,7 +43391,11 @@
       </c>
       <c r="H418" s="9" t="inlineStr"/>
       <c r="I418" s="9" t="inlineStr"/>
-      <c r="J418" s="9" t="inlineStr"/>
+      <c r="J418" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K418" s="9" t="inlineStr"/>
       <c r="L418" s="9" t="n">
         <v>100</v>
@@ -44299,7 +44343,11 @@
       </c>
       <c r="H432" s="9" t="inlineStr"/>
       <c r="I432" s="9" t="inlineStr"/>
-      <c r="J432" s="9" t="inlineStr"/>
+      <c r="J432" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K432" s="9" t="inlineStr"/>
       <c r="L432" s="9" t="n">
         <v>100</v>
@@ -44363,7 +44411,11 @@
       </c>
       <c r="H433" s="9" t="inlineStr"/>
       <c r="I433" s="9" t="inlineStr"/>
-      <c r="J433" s="9" t="inlineStr"/>
+      <c r="J433" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K433" s="9" t="inlineStr"/>
       <c r="L433" s="9" t="n">
         <v>100</v>
@@ -44427,7 +44479,11 @@
       </c>
       <c r="H434" s="9" t="inlineStr"/>
       <c r="I434" s="9" t="inlineStr"/>
-      <c r="J434" s="9" t="inlineStr"/>
+      <c r="J434" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K434" s="9" t="inlineStr"/>
       <c r="L434" s="9" t="n">
         <v>100</v>
@@ -44628,7 +44684,11 @@
       </c>
       <c r="H437" s="9" t="inlineStr"/>
       <c r="I437" s="9" t="inlineStr"/>
-      <c r="J437" s="9" t="inlineStr"/>
+      <c r="J437" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K437" s="9" t="inlineStr"/>
       <c r="L437" s="9" t="n">
         <v>100</v>
@@ -45102,7 +45162,11 @@
       </c>
       <c r="H444" s="9" t="inlineStr"/>
       <c r="I444" s="9" t="inlineStr"/>
-      <c r="J444" s="9" t="inlineStr"/>
+      <c r="J444" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K444" s="9" t="inlineStr"/>
       <c r="L444" s="9" t="n">
         <v>100</v>
@@ -45370,7 +45434,11 @@
       </c>
       <c r="H448" s="9" t="inlineStr"/>
       <c r="I448" s="9" t="inlineStr"/>
-      <c r="J448" s="9" t="inlineStr"/>
+      <c r="J448" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K448" s="9" t="inlineStr"/>
       <c r="L448" s="9" t="n">
         <v>100</v>
@@ -45434,7 +45502,11 @@
       </c>
       <c r="H449" s="9" t="inlineStr"/>
       <c r="I449" s="9" t="inlineStr"/>
-      <c r="J449" s="9" t="inlineStr"/>
+      <c r="J449" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K449" s="9" t="inlineStr"/>
       <c r="L449" s="9" t="n">
         <v>81.25</v>
@@ -45498,7 +45570,11 @@
       </c>
       <c r="H450" s="9" t="inlineStr"/>
       <c r="I450" s="9" t="inlineStr"/>
-      <c r="J450" s="9" t="inlineStr"/>
+      <c r="J450" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K450" s="9" t="inlineStr"/>
       <c r="L450" s="9" t="n">
         <v>81.25</v>
@@ -45562,7 +45638,11 @@
       </c>
       <c r="H451" s="9" t="inlineStr"/>
       <c r="I451" s="9" t="inlineStr"/>
-      <c r="J451" s="9" t="inlineStr"/>
+      <c r="J451" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K451" s="9" t="inlineStr"/>
       <c r="L451" s="9" t="n">
         <v>62.5</v>
@@ -46017,7 +46097,11 @@
       </c>
       <c r="H457" s="9" t="inlineStr"/>
       <c r="I457" s="9" t="inlineStr"/>
-      <c r="J457" s="9" t="inlineStr"/>
+      <c r="J457" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K457" s="9" t="inlineStr"/>
       <c r="L457" s="9" t="n">
         <v>0</v>
@@ -46091,7 +46175,11 @@
       </c>
       <c r="H458" s="9" t="inlineStr"/>
       <c r="I458" s="9" t="inlineStr"/>
-      <c r="J458" s="9" t="inlineStr"/>
+      <c r="J458" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K458" s="9" t="inlineStr"/>
       <c r="L458" s="9" t="n">
         <v>0</v>
@@ -46243,7 +46331,11 @@
       </c>
       <c r="H460" s="9" t="inlineStr"/>
       <c r="I460" s="9" t="inlineStr"/>
-      <c r="J460" s="9" t="inlineStr"/>
+      <c r="J460" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K460" s="9" t="inlineStr"/>
       <c r="L460" s="9" t="n">
         <v>25</v>
@@ -46385,7 +46477,11 @@
       </c>
       <c r="H462" s="9" t="inlineStr"/>
       <c r="I462" s="9" t="inlineStr"/>
-      <c r="J462" s="9" t="inlineStr"/>
+      <c r="J462" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K462" s="9" t="inlineStr"/>
       <c r="L462" s="9" t="n">
         <v>0</v>
@@ -46459,7 +46555,11 @@
       </c>
       <c r="H463" s="9" t="inlineStr"/>
       <c r="I463" s="9" t="inlineStr"/>
-      <c r="J463" s="9" t="inlineStr"/>
+      <c r="J463" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K463" s="9" t="inlineStr"/>
       <c r="L463" s="9" t="n">
         <v>0</v>
@@ -46533,7 +46633,11 @@
       </c>
       <c r="H464" s="9" t="inlineStr"/>
       <c r="I464" s="9" t="inlineStr"/>
-      <c r="J464" s="9" t="inlineStr"/>
+      <c r="J464" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K464" s="9" t="inlineStr"/>
       <c r="L464" s="9" t="n">
         <v>0</v>
@@ -47066,7 +47170,11 @@
       </c>
       <c r="H471" s="9" t="inlineStr"/>
       <c r="I471" s="9" t="inlineStr"/>
-      <c r="J471" s="9" t="inlineStr"/>
+      <c r="J471" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K471" s="9" t="inlineStr"/>
       <c r="L471" s="9" t="n">
         <v>25</v>
@@ -47198,7 +47306,11 @@
       </c>
       <c r="H473" s="9" t="inlineStr"/>
       <c r="I473" s="9" t="inlineStr"/>
-      <c r="J473" s="9" t="inlineStr"/>
+      <c r="J473" s="9" t="inlineStr">
+        <is>
+          <t>กทม.</t>
+        </is>
+      </c>
       <c r="K473" s="9" t="inlineStr"/>
       <c r="L473" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
Wording: refine status-group labels (construction zone, physical constraint, external agency, temporary measure, in progress)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9111,7 +9111,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ติดข้อจำกัดหน่วยงานอื่น</t>
+          <t>ข้อจำกัดหน่วยงานภายนอก</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -9341,7 +9341,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -9387,7 +9387,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>มาตรการชั่วคราว</t>
+          <t>ใช้มาตรการชั่วคราว</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>มาตรการชั่วคราว</t>
+          <t>ใช้มาตรการชั่วคราว</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>กำลังดำเนินการ</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -36003,7 +36003,7 @@
       </c>
       <c r="V315" t="inlineStr">
         <is>
-          <t>ติดข้อจำกัดหน่วยงานอื่น</t>
+          <t>ข้อจำกัดหน่วยงานภายนอก</t>
         </is>
       </c>
     </row>
@@ -36735,7 +36735,7 @@
       </c>
       <c r="V325" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -36818,7 +36818,7 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -37118,7 +37118,7 @@
       </c>
       <c r="V330" t="inlineStr">
         <is>
-          <t>มาตรการชั่วคราว</t>
+          <t>ใช้มาตรการชั่วคราว</t>
         </is>
       </c>
     </row>
@@ -41922,7 +41922,7 @@
       </c>
       <c r="V396" t="inlineStr">
         <is>
-          <t>กำลังดำเนินการ</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
     </row>
@@ -45826,7 +45826,7 @@
       </c>
       <c r="V453" t="inlineStr">
         <is>
-          <t>มาตรการชั่วคราว</t>
+          <t>ใช้มาตรการชั่วคราว</t>
         </is>
       </c>
     </row>
@@ -45904,7 +45904,7 @@
       </c>
       <c r="V454" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -45983,7 +45983,7 @@
       </c>
       <c r="V455" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -46061,7 +46061,7 @@
       </c>
       <c r="V456" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
     </row>
@@ -46217,7 +46217,7 @@
       </c>
       <c r="V458" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -46295,7 +46295,7 @@
       </c>
       <c r="V459" t="inlineStr">
         <is>
-          <t>มาตรการชั่วคราว</t>
+          <t>ใช้มาตรการชั่วคราว</t>
         </is>
       </c>
     </row>
@@ -46441,7 +46441,7 @@
       </c>
       <c r="V461" t="inlineStr">
         <is>
-          <t>กำลังดำเนินการ</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
     </row>
@@ -46597,7 +46597,7 @@
       </c>
       <c r="V463" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
     </row>
@@ -46675,7 +46675,7 @@
       </c>
       <c r="V464" t="inlineStr">
         <is>
-          <t>ข้อจำกัดกายภาพ</t>
+          <t>ข้อจำกัดทางกายภาพ</t>
         </is>
       </c>
     </row>
@@ -46832,7 +46832,7 @@
       </c>
       <c r="V466" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>
@@ -46910,7 +46910,7 @@
       </c>
       <c r="V467" t="inlineStr">
         <is>
-          <t>ติดก่อสร้างรถไฟฟ้า</t>
+          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: separate Toyota Bhumibhat U-turn from Vejkarunrasm Hospital U-turn (approx coords ~120m apart, pending field verification) — unique locations now 156 = 127+77-48
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9022,7 +9022,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -9943,10 +9942,10 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>13.85579832</v>
+        <v>13.8569</v>
       </c>
       <c r="J22" t="n">
-        <v>100.8527928</v>
+        <v>100.8528</v>
       </c>
     </row>
     <row r="23">
@@ -15120,7 +15119,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -46663,10 +46661,10 @@
         <v>0</v>
       </c>
       <c r="S464" s="9" t="n">
-        <v>13.85579832</v>
+        <v>13.8569</v>
       </c>
       <c r="T464" s="9" t="n">
-        <v>100.8527928</v>
+        <v>100.8528</v>
       </c>
       <c r="U464" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix: dedupe corridors sheet (72->47 rows) — persistent corridors KPI now correctly 25 matching hero/README
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1460,7 +1460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1484,6 +1484,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -1491,6 +1492,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -3713,6 +3715,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
@@ -3720,6 +3723,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
@@ -3779,1206 +3783,6 @@
       <c r="L54" s="8" t="inlineStr">
         <is>
           <t>sample_names</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="B55" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="C55" s="9" t="n">
-        <v>13.77902180857143</v>
-      </c>
-      <c r="D55" s="9" t="n">
-        <v>100.5092926857143</v>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>ดุสิต</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>ถนนสามเสน</t>
-        </is>
-      </c>
-      <c r="H55" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I55" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J55" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K55" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L55" s="9" t="inlineStr">
-        <is>
-          <t>แยกวชิระ  (ถนนสามเสน - ถนนสุโขทัย); แยกการเรือน (ถนนราชวิถี - ถนนราชสีมา); แยกซังฮี้ (ถนนสามเสน - ถนนราชวิถี)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="B56" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="C56" s="9" t="n">
-        <v>13.75676817428571</v>
-      </c>
-      <c r="D56" s="9" t="n">
-        <v>100.4832968857143</v>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>บางกอกน้อย</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนเหนือ</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="inlineStr">
-        <is>
-          <t>ถนนอรุณอมรินทร์</t>
-        </is>
-      </c>
-      <c r="H56" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I56" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J56" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K56" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L56" s="9" t="inlineStr">
-        <is>
-          <t>แยกศิริราช  (ถนนอรุณอมรินทร์ - ถนนพรานนก; แยกศิริราช; คอขวดบริเวณหน้าโรงพยาบาลศิริราช ถนนอรุณอ</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B57" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="C57" s="9" t="n">
-        <v>13.74584893666667</v>
-      </c>
-      <c r="D57" s="9" t="n">
-        <v>100.5321741333333</v>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>ปทุมวัน</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพใต้</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพระรามที่ 1</t>
-        </is>
-      </c>
-      <c r="H57" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I57" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="J57" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K57" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L57" s="9" t="inlineStr">
-        <is>
-          <t>แยกปทุมวัน; ถนนพระรามที่ 1  หน้าห้างสรรพสินค้าสยามเซ; หน้าห้างสรรพสินค้ามาบุญครอง (MBK Center)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="n">
-        <v>39</v>
-      </c>
-      <c r="B58" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="C58" s="9" t="n">
-        <v>13.67426480166667</v>
-      </c>
-      <c r="D58" s="9" t="n">
-        <v>100.4261541166667</v>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>บางบอน</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนใต้</t>
-        </is>
-      </c>
-      <c r="G58" s="9" t="inlineStr">
-        <is>
-          <t>ถนนเอกชัย</t>
-        </is>
-      </c>
-      <c r="H58" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I58" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J58" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K58" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L58" s="9" t="inlineStr">
-        <is>
-          <t>สามแยกบางบอน และสามแยกบางบอน 1  ถนนเอกชั; คอขวดหน้าตลาดบางบอน ถนนเอกชัย; แยกบางบอน</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B59" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="C59" s="9" t="n">
-        <v>13.757871816</v>
-      </c>
-      <c r="D59" s="9" t="n">
-        <v>100.5346068</v>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>ราชเทวี</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G59" s="9" t="inlineStr">
-        <is>
-          <t>ถนนศรีอยุธยา /ถนนพญาไท</t>
-        </is>
-      </c>
-      <c r="H59" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I59" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J59" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K59" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L59" s="9" t="inlineStr">
-        <is>
-          <t>แยกพญาไท (ถนนพญาไท - ถนนศรีอยุธยา); แยกพญาไท; จุดกลับรถใกล้แยกพญาไท</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="B60" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="C60" s="9" t="n">
-        <v>13.7714682</v>
-      </c>
-      <c r="D60" s="9" t="n">
-        <v>100.4833052</v>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>บางกอกน้อย</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนเหนือ</t>
-        </is>
-      </c>
-      <c r="G60" s="9" t="inlineStr">
-        <is>
-          <t>ถนนสมเด็จพระปิ่นเกล้า</t>
-        </is>
-      </c>
-      <c r="H60" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I60" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J60" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K60" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L60" s="9" t="inlineStr">
-        <is>
-          <t>สี่แยกบรมราชชนนี; ป้ายรถประจำทางตรงข้ามห้างสรรพสินค้าพาต้า; คอขวดบริเวณตรงข้ามห้างสรรพสินค้าพาต้าปิ่</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B61" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="C61" s="9" t="n">
-        <v>13.7446348</v>
-      </c>
-      <c r="D61" s="9" t="n">
-        <v>100.5408396</v>
-      </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>ปทุมวัน</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพใต้</t>
-        </is>
-      </c>
-      <c r="G61" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพระรามที่ 1 /ถนนราชดำริ</t>
-        </is>
-      </c>
-      <c r="H61" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I61" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="J61" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K61" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L61" s="9" t="inlineStr">
-        <is>
-          <t>หน้าโรงเรียนมาแตร์ เดอี  (ถนนเพลินจิต); หน้าห้างเซนทรัลเวิลด์ ข้างศาลพระตรีมูรติ; แยกราชประสงค์</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B62" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C62" s="9" t="n">
-        <v>13.79848936</v>
-      </c>
-      <c r="D62" s="9" t="n">
-        <v>100.55131665</v>
-      </c>
-      <c r="E62" s="9" t="inlineStr">
-        <is>
-          <t>จตุจักร</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพเหนือ</t>
-        </is>
-      </c>
-      <c r="G62" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพหลโยธิน</t>
-        </is>
-      </c>
-      <c r="H62" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I62" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J62" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K62" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L62" s="9" t="inlineStr">
-        <is>
-          <t>บริเวณหน้าตลาดนัดจตุจักร; บริเวณแยกกำแพงเพชร - ห้าแยกลาดพร้าว (ถนน; คอขวดบริเวณหน้าตลาดนัดจตุจักร</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C63" s="9" t="n">
-        <v>13.79910575</v>
-      </c>
-      <c r="D63" s="9" t="n">
-        <v>100.533908</v>
-      </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>ดุสิต</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G63" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพระรามที่ 6</t>
-        </is>
-      </c>
-      <c r="H63" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I63" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J63" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K63" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L63" s="9" t="inlineStr">
-        <is>
-          <t>แยกถนนพระราม 6 ตัดถนนเตชวะนิช; คอขวดถนนพระรามหกตัดใหม่ (อุโมงค์ทางลอดสะ; คอขวดแยกวัดสะพานสูง</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B64" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C64" s="9" t="n">
-        <v>13.75536</v>
-      </c>
-      <c r="D64" s="9" t="n">
-        <v>100.5414655</v>
-      </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>ราชเทวี</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G64" s="9" t="inlineStr">
-        <is>
-          <t>ถนนราชปรารภ</t>
-        </is>
-      </c>
-      <c r="H64" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I64" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J64" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K64" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L64" s="9" t="inlineStr">
-        <is>
-          <t>ถนนจตุรทิศ (หน้าโรงพยาบาลพญาไท 1); แยกมักกะสัน; แยกมักกะสัน</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B65" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C65" s="9" t="n">
-        <v>13.7474072225</v>
-      </c>
-      <c r="D65" s="9" t="n">
-        <v>100.521103325</v>
-      </c>
-      <c r="E65" s="9" t="inlineStr">
-        <is>
-          <t>ปทุมวัน</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพใต้</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพระรามที่ 1</t>
-        </is>
-      </c>
-      <c r="H65" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I65" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J65" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K65" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L65" s="9" t="inlineStr">
-        <is>
-          <t>สะพานกษัตริย์ศึก (ถนนพระรามที่ 1); ถนนบรรทัดทอง; ป้ายรถประจำทางตรงข้ามวัดชำนิหัตถการ ถนนพ</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B66" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C66" s="9" t="n">
-        <v>13.6613605</v>
-      </c>
-      <c r="D66" s="9" t="n">
-        <v>100.404371</v>
-      </c>
-      <c r="E66" s="9" t="inlineStr">
-        <is>
-          <t>บางบอน</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนใต้</t>
-        </is>
-      </c>
-      <c r="G66" s="9" t="inlineStr">
-        <is>
-          <t>ถนนเอกชัย</t>
-        </is>
-      </c>
-      <c r="H66" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I66" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J66" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K66" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L66" s="9" t="inlineStr">
-        <is>
-          <t>ถนนเอกชัย (ฝั่งเลขคู่)  เลี้ยงซ้ายเข้า ถ; ถนนกาญจนาภิเษก แขวงบางบอนเหนือ แขวงคลองบ; จุดกลับรถหน้าไปรษณีย์ย่อยบางบอน ถนนเอกชั</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B67" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C67" s="9" t="n">
-        <v>13.8124435</v>
-      </c>
-      <c r="D67" s="9" t="n">
-        <v>100.726485</v>
-      </c>
-      <c r="E67" s="9" t="inlineStr">
-        <is>
-          <t>มีนบุรี</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพตะวันออก</t>
-        </is>
-      </c>
-      <c r="G67" s="9" t="inlineStr">
-        <is>
-          <t>ถนนสีหบุรานุกิจ</t>
-        </is>
-      </c>
-      <c r="H67" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I67" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J67" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K67" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L67" s="9" t="inlineStr">
-        <is>
-          <t>หน้าตลาดนัดจตุจักร 2 (มีนบุรี)  (ถนนสีหบ; ตลาดนัดจตุจักร 2 (มีนบุรี)  (ถนนสุวินทวง; ป้ายรถประจำทางหน้าธนาคารออมสิน ถนนสีหบุร</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B68" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C68" s="9" t="n">
-        <v>13.83055333333333</v>
-      </c>
-      <c r="D68" s="9" t="n">
-        <v>100.5391973333333</v>
-      </c>
-      <c r="E68" s="9" t="inlineStr">
-        <is>
-          <t>จตุจักร</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพเหนือ</t>
-        </is>
-      </c>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>ถนนประชานุกูล</t>
-        </is>
-      </c>
-      <c r="H68" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I68" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J68" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K68" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L68" s="9" t="inlineStr">
-        <is>
-          <t>บริเวณทางลงทางด่วนประชานุกูล (ครอบคลุมถึ; จุดกลับรถใต้สะพานข้ามแยกประชานุกูล; จุดกลับรถใต้สะพานข้ามแยกประชานุกูล</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B69" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C69" s="9" t="n">
-        <v>13.81387952</v>
-      </c>
-      <c r="D69" s="9" t="n">
-        <v>100.5600307333333</v>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>จตุจักร</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพเหนือ</t>
-        </is>
-      </c>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>ถนนลาดพร้าว</t>
-        </is>
-      </c>
-      <c r="H69" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I69" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J69" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K69" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L69" s="9" t="inlineStr">
-        <is>
-          <t>บริเวณสะพานข้ามแยกลาดพร้าว (มุ่งหน้าไปดิ; คอขวดปากทางลาดพร้าว (ช่วงโค้งถนนลาดพร้าว; คอขวดปากทางลาดพร้าว (โค้งถนนลาดพร้าวก่อน</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B70" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C70" s="9" t="n">
-        <v>13.79744696</v>
-      </c>
-      <c r="D70" s="9" t="n">
-        <v>100.5458070666667</v>
-      </c>
-      <c r="E70" s="9" t="inlineStr">
-        <is>
-          <t>จตุจักร</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพเหนือ</t>
-        </is>
-      </c>
-      <c r="G70" s="9" t="inlineStr">
-        <is>
-          <t>ถนนกำแพงเพชร</t>
-        </is>
-      </c>
-      <c r="H70" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I70" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J70" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K70" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L70" s="9" t="inlineStr">
-        <is>
-          <t>บริเวณหน้าตลาดต้นไม้; คอขวดบริเวณหน้าตลาดต้นไม้; คอขวดบริเวณหน้าตลาดต้นไม้</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B71" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C71" s="9" t="n">
-        <v>13.76262892666667</v>
-      </c>
-      <c r="D71" s="9" t="n">
-        <v>100.5239707333333</v>
-      </c>
-      <c r="E71" s="9" t="inlineStr">
-        <is>
-          <t>ราชเทวี</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G71" s="9" t="inlineStr">
-        <is>
-          <t>ถนนศรีอยุธยา /ถนนสวรรคโลก</t>
-        </is>
-      </c>
-      <c r="H71" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I71" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J71" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K71" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L71" s="9" t="inlineStr">
-        <is>
-          <t>แยกศรีอยุธยา (ถนนพระรามที่ 6 - ถนนศรีอยุ; แยกเสาวนี; แยกเสาวนี</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B72" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C72" s="9" t="n">
-        <v>13.79233549333334</v>
-      </c>
-      <c r="D72" s="9" t="n">
-        <v>100.5359064666667</v>
-      </c>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>ดุสิต</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G72" s="9" t="inlineStr">
-        <is>
-          <t>ถนนประดิพัทธ์ /ถนนเทอดดำริ</t>
-        </is>
-      </c>
-      <c r="H72" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I72" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J72" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K72" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L72" s="9" t="inlineStr">
-        <is>
-          <t>แยกประดิพัทธ์ (ถนนพระรามที่ 6 - ถนนประดิ; แยกเทอดดำริ; แยกเทอดดำริ</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B73" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C73" s="9" t="n">
-        <v>13.791062</v>
-      </c>
-      <c r="D73" s="9" t="n">
-        <v>100.5488446666666</v>
-      </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>พญาไท</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพกลาง</t>
-        </is>
-      </c>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพหลโยธิน</t>
-        </is>
-      </c>
-      <c r="H73" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I73" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J73" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K73" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L73" s="9" t="inlineStr">
-        <is>
-          <t>แยกสะพานควาย (ถนนพหลโยธิน - ถนนประดิพัทธ; คอขวดหน้าห้างฯ บิ๊กซี สะพานควาย ถนนพหลโย; คอขวดหน้าห้างสรรพสินค้าบิ๊กซีสะพานควาย ถ</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B74" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C74" s="9" t="n">
-        <v>13.78197114666667</v>
-      </c>
-      <c r="D74" s="9" t="n">
-        <v>100.6828355333333</v>
-      </c>
-      <c r="E74" s="9" t="inlineStr">
-        <is>
-          <t>สะพานสูง</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพตะวันออก</t>
-        </is>
-      </c>
-      <c r="G74" s="9" t="inlineStr">
-        <is>
-          <t>ถนนรามคำแหง</t>
-        </is>
-      </c>
-      <c r="H74" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I74" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J74" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K74" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L74" s="9" t="inlineStr">
-        <is>
-          <t>แยกคลองเจ็ก ถนนรามคำแหง  (ศูนย์ควบคุมและ; แยกคลองเจ็ก ถนนรามคำแหง; แยกคลองเจ็ก ถนนรามคำแหง</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B75" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C75" s="9" t="n">
-        <v>13.92354555333333</v>
-      </c>
-      <c r="D75" s="9" t="n">
-        <v>100.6250466666667</v>
-      </c>
-      <c r="E75" s="9" t="inlineStr">
-        <is>
-          <t>สายไหม</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพเหนือ</t>
-        </is>
-      </c>
-      <c r="G75" s="9" t="inlineStr">
-        <is>
-          <t>ถนนพหลโยธิน</t>
-        </is>
-      </c>
-      <c r="H75" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I75" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J75" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K75" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L75" s="9" t="inlineStr">
-        <is>
-          <t>แยก รร. นายเรืออากาศ (ค.ป.อ.) (ถนนพหลโยธ; แยก คปอ.; แยก คปอ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="9" t="n">
-        <v>29</v>
-      </c>
-      <c r="B76" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C76" s="9" t="n">
-        <v>13.74295633333333</v>
-      </c>
-      <c r="D76" s="9" t="n">
-        <v>100.5494016666666</v>
-      </c>
-      <c r="E76" s="9" t="inlineStr">
-        <is>
-          <t>ปทุมวัน</t>
-        </is>
-      </c>
-      <c r="F76" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพใต้</t>
-        </is>
-      </c>
-      <c r="G76" s="9" t="inlineStr">
-        <is>
-          <t>ถนนเพลินจิต</t>
-        </is>
-      </c>
-      <c r="H76" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I76" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J76" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K76" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L76" s="9" t="inlineStr">
-        <is>
-          <t>ใต้ทางด่วนเพลินจิตมุ่งหน้าถนนเพลินจิต  (; คอขวดบริเวณด่านเก็บค่าผ่านทางพิเศษเพลินจ; ปรับการจัดการจราจรถนนพระรามที่ 1 แยกเพลิ</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B77" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C77" s="9" t="n">
-        <v>13.737275</v>
-      </c>
-      <c r="D77" s="9" t="n">
-        <v>100.4940866666667</v>
-      </c>
-      <c r="E77" s="9" t="inlineStr">
-        <is>
-          <t>ธนบุรี</t>
-        </is>
-      </c>
-      <c r="F77" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนเหนือ</t>
-        </is>
-      </c>
-      <c r="G77" s="9" t="inlineStr">
-        <is>
-          <t>ซอยอรุณอมรินทร์ 4</t>
-        </is>
-      </c>
-      <c r="H77" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I77" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J77" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K77" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L77" s="9" t="inlineStr">
-        <is>
-          <t>ซอยอรุณอมรินทร์ 4 และถนนอรุณอมรินทร์บรรจ; คอขวดโรงเรียนซางตาครู้สคอนแวนต์ ถนนเทศบา; คอขวดโรงเรียนซางตาครู้สคอนแวนต์ ถนนเทศบา</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B78" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C78" s="9" t="n">
-        <v>13.71139933333333</v>
-      </c>
-      <c r="D78" s="9" t="n">
-        <v>100.609978</v>
-      </c>
-      <c r="E78" s="9" t="inlineStr">
-        <is>
-          <t>สวนหลวง</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="inlineStr">
-        <is>
-          <t>กรุงเทพใต้</t>
-        </is>
-      </c>
-      <c r="G78" s="9" t="inlineStr">
-        <is>
-          <t>ถนนอ่อนนุช</t>
-        </is>
-      </c>
-      <c r="H78" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I78" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J78" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K78" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L78" s="9" t="inlineStr">
-        <is>
-          <t>แยกอ่อนนุช 17 (ถนนอ่อนนุช - อ่อนนุช ซอย ; แยกอ่อนนุช 17 (ถนนอ่อนนุช - อ่อนนุช ซอย ; แยกอ่อนนุช 17 (ถนนอ่อนนุช-อ่อนนุช ซอย 17</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B79" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C79" s="9" t="n">
-        <v>13.712633</v>
-      </c>
-      <c r="D79" s="9" t="n">
-        <v>100.428358</v>
-      </c>
-      <c r="E79" s="9" t="inlineStr">
-        <is>
-          <t>ภาษีเจริญ</t>
-        </is>
-      </c>
-      <c r="F79" s="9" t="inlineStr">
-        <is>
-          <t>กรุงธนใต้</t>
-        </is>
-      </c>
-      <c r="G79" s="9" t="inlineStr">
-        <is>
-          <t>ถนนเพชรเกษม /ถนนพุทธมณฑลสาย 1</t>
-        </is>
-      </c>
-      <c r="H79" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I79" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J79" s="9" t="inlineStr">
-        <is>
-          <t>[2566, 2567, 2568]</t>
-        </is>
-      </c>
-      <c r="K79" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L79" s="9" t="inlineStr">
-        <is>
-          <t>แยกถนนเพชรเกษม-พุทธมณฑล สาย 1  (ถนนเพชรเ; แยกถนนเพชรเกษม-พุทธมณฑลสาย 1; แยกถนนเพชรเกษม-พุทธมณฑลสาย 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize status labels per data values across all pages: 0% = Tid Panha Upasak (blocked), 1-99% = In Progress, 100% = Complete; unresolved section now 8 blocked + 15 in-progress with raw xlsx remarks
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -7855,12 +7855,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>สถานะล่าสุด</t>
+          <t>สถานะ</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>กลุ่มสถานะ</t>
+          <t>หมายเหตุ</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7890,37 +7890,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>แยกลาซาลตัดแบริ่ง</t>
+          <t>บริเวณทางเชื่อมระหว่างมอเตอร์เวย์กับถนนพระราม 9</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>บางนา</t>
+          <t>สวนหลวง</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>กทม.</t>
+          <t>ทล.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>81.25</v>
+        <v>0</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>เป็นพื้นทีรับผิดชอบของกรมทางหลวง</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>13.660765</v>
+        <v>13.742533</v>
       </c>
       <c r="J4" t="n">
-        <v>100.624963</v>
+        <v>100.63775</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -7934,17 +7934,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>แยกศรีนครินทร์-ลาซาล (แยกศรีลาซาล)</t>
+          <t>คอขวดถนนสามเสนช่วงก่อนถึงแยกซังฮี้ ทางทิศใต้</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>บางนา</t>
+          <t>ดุสิต</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7953,27 +7953,27 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>81.25</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ติดแนวก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>13.65622</v>
+        <v>13.77983333</v>
       </c>
       <c r="J5" t="n">
-        <v>100.642369</v>
+        <v>100.5091389</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>กรุงเทพใต้</t>
+          <t>กรุงเทพกลาง</t>
         </is>
       </c>
     </row>
@@ -7983,17 +7983,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>แยกหน้าทางเข้าโรงเรียนปาณยาพัฒนาการ</t>
+          <t>แยกซังฮี้</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>สวนหลวง</t>
+          <t>ดุสิต</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -8002,27 +8002,27 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ติดแนวก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>13.737036</v>
+        <v>13.778386</v>
       </c>
       <c r="J6" t="n">
-        <v>100.626139</v>
+        <v>100.508418</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>กรุงเทพใต้</t>
+          <t>กรุงเทพกลาง</t>
         </is>
       </c>
     </row>
@@ -8032,22 +8032,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>บริเวณทางเชื่อมระหว่างมอเตอร์เวย์กับถนนพระราม 9</t>
+          <t>จุดกลับรถใกล้แยกพญาไท</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>สวนหลวง</t>
+          <t>ราชเทวี</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ทล.</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -8055,23 +8055,23 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>อยู่ในความรับผิดชอบ ทล. (กรมทางหลวง)</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>นอกอำนาจ กทม.</t>
+          <t>ติดแนวก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>13.742533</v>
+        <v>13.75775</v>
       </c>
       <c r="J7" t="n">
-        <v>100.63775</v>
+        <v>100.5349167</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>กรุงเทพใต้</t>
+          <t>กรุงเทพกลาง</t>
         </is>
       </c>
     </row>
@@ -8081,17 +8081,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>คอขวดโรงเรียนซางตาครู้สคอนแวนต์ ถนนเทศบาลสาย 1 (ซอยอรุณอมรินทร์ 4)</t>
+          <t>แยกหมอเหล็ง</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ธนบุรี</t>
+          <t>ราชเทวี</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8100,27 +8100,27 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ใช้มาตรการชั่วคราว</t>
+          <t>ติดแนวก่อสร้างรถไฟฟ้า</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>13.737245</v>
+        <v>13.7559668535117</v>
       </c>
       <c r="J8" t="n">
-        <v>100.49404</v>
+        <v>100.542319210583</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>กรุงธนเหนือ</t>
+          <t>กรุงเทพกลาง</t>
         </is>
       </c>
     </row>
@@ -8130,17 +8130,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>คอขวดถนนสามเสนช่วงก่อนถึงแยกซังฮี้ ทางทิศใต้</t>
+          <t>จุดกลับรถหน้าโรงพยาบาลเวชการุณย์รัศมิ์</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ดุสิต</t>
+          <t>หนองจอก</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -8153,23 +8153,23 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ติดแนวก่อสร้างรถไฟฟ้าสายสีม่วง รอคืนผิวจราจรจาก รฟม.</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
+          <t>ความกว้างถนนไม่เพียงพอให้ปรับช่องจราจร</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>13.77983333</v>
+        <v>13.8558359592258</v>
       </c>
       <c r="J9" t="n">
-        <v>100.5091389</v>
+        <v>100.858545070494</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>กรุงเทพกลาง</t>
+          <t>กรุงเทพตะวันออก</t>
         </is>
       </c>
     </row>
@@ -8179,17 +8179,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>แยกซังฮี้</t>
+          <t>จุดกลับรถหน้าโตโยต้าภูมิพัฒนา</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ดุสิต</t>
+          <t>หนองจอก</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8202,23 +8202,23 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ติดแนวก่อสร้างรถไฟฟ้าสายสีม่วง รอคืนผิวจราจรจาก รฟม.</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
+          <t>ความกว้างถนนไม่เพียงพอให้ปรับช่องจราจร</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>13.778386</v>
+        <v>13.8557481105835</v>
       </c>
       <c r="J10" t="n">
-        <v>100.508418</v>
+        <v>100.853164957125</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>กรุงเทพกลาง</t>
+          <t>กรุงเทพตะวันออก</t>
         </is>
       </c>
     </row>
@@ -8228,22 +8228,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2567</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>จุดกลับรถใกล้แยกพญาไท</t>
+          <t>แยกต่างระดับราชพฤกษ์ - รัชดาภิเษก</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ราชเทวี</t>
+          <t>ธนบุรี</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>กทม.</t>
+          <t>ทช.</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -8251,23 +8251,23 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ติดแนวก่อสร้างรถไฟฟ้าสายสีส้ม รอคืนผิวจราจรจาก รฟม.</t>
+          <t>ติดปัญหาอุปสรรค</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
+          <t>ความรับผิดชอบของกรมทางหลวงชนบท</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>13.75775</v>
+        <v>13.7154111</v>
       </c>
       <c r="J11" t="n">
-        <v>100.5349167</v>
+        <v>100.4782633</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>กรุงเทพกลาง</t>
+          <t>กรุงธนเหนือ</t>
         </is>
       </c>
     </row>
@@ -8277,17 +8277,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>แยกกำแพงเพชร 7-อโศกดินแดง</t>
+          <t>คอขวดโรงเรียนซางตาครู้สคอนแวนต์ ถนนเทศบาลสาย 1 (ซอยอรุณอมรินทร์ 4)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ราชเทวี</t>
+          <t>ธนบุรี</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8300,23 +8300,23 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ (สัญญาณไฟ adaptive งบปี 2569 อยู่ระหว่างอนุมัติจ้าง)</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>ประสานตำรวจแล้ว</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>13.74999</v>
+        <v>13.737245</v>
       </c>
       <c r="J12" t="n">
-        <v>100.563632</v>
+        <v>100.49404</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>กรุงเทพกลาง</t>
+          <t>กรุงธนเหนือ</t>
         </is>
       </c>
     </row>
@@ -8331,7 +8331,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>แยกหมอเหล็ง</t>
+          <t>แยกกำแพงเพชร 7-อโศกดินแดง</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -8345,23 +8345,23 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>ติดแนวก่อสร้างรถไฟฟ้าสายสีส้ม รอคืนผิวจราจรจาก รฟม.</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>พื้นที่ก่อสร้างรถไฟฟ้า</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>13.7559668535117</v>
+        <v>13.74999</v>
       </c>
       <c r="J13" t="n">
-        <v>100.542319210583</v>
+        <v>100.563632</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -8398,12 +8398,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>ประสานตำรวจกวดขันวินัยจราจรแล้ว</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ใช้มาตรการชั่วคราว</t>
+          <t>ประสานตำรวจแล้ว</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -8424,12 +8424,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>แยกใต้ทางด่วนพระราม 9 (แยก RCA)</t>
+          <t>คอขวดทางขึ้นสะพานข้ามคลองแสนแสบ ด้านถนนเพชรบุรี</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8443,7 +8443,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -8452,14 +8452,14 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ</t>
+          <t>สำนักการโยธาอยู่ระหว่างการก่อสร้าง</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>13.7527203</v>
+        <v>13.74208333</v>
       </c>
       <c r="J15" t="n">
-        <v>100.5743538</v>
+        <v>100.59625</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -8473,12 +8473,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>คอขวดทางขึ้นสะพานข้ามคลองแสนแสบ ด้านถนนเพชรบุรี</t>
+          <t>แยกจุดใต้ทางด่วนพระราม 9 (หน้าโรงพยาบาลปิยะเวท)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>สนย.อยู่ระหว่างก่อสร้างปรับปรุงสะพาน</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -8505,10 +8505,10 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>13.74208333</v>
+        <v>13.7543877</v>
       </c>
       <c r="J16" t="n">
-        <v>100.59625</v>
+        <v>100.5796209</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -8522,17 +8522,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>แยกจุดใต้ทางด่วนพระราม 9 (หน้าโรงพยาบาลปิยะเวท)</t>
+          <t>จุดกลับรถหน้าหมู่บ้านศรีประจักษ์ ถนนรามคำแหง</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ห้วยขวาง</t>
+          <t>สะพานสูง</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -8545,23 +8545,18 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>อยู่ระหว่างดำเนินการ (สัญญาณไฟ adaptive งบปี 2569 อยู่ระหว่างอนุมัติจ้าง)</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
           <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>13.7543877</v>
+        <v>13.787472</v>
       </c>
       <c r="J17" t="n">
-        <v>100.5796209</v>
+        <v>100.6927</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>กรุงเทพกลาง</t>
+          <t>กรุงเทพตะวันออก</t>
         </is>
       </c>
     </row>
@@ -8571,17 +8566,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2568</t>
+          <t>2567/2568</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>จุดกลับรถหน้าโรงพยาบาลเวชการุณย์รัศมิ์</t>
+          <t>จุดกลับรถหน้าหมู่บ้านสัมมากร ประตู 2 ถนนรามคำแหง</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>หนองจอก</t>
+          <t>สะพานสูง</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -8590,23 +8585,18 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ความกว้างถนนไม่เพียงพอให้ปรับช่องจราจร</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>ข้อจำกัดทางกายภาพ</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>13.8558359592258</v>
+        <v>13.777225</v>
       </c>
       <c r="J18" t="n">
-        <v>100.858545070494</v>
+        <v>100.674031</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -8625,12 +8615,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>จุดกลับรถหน้าโตโยต้าภูมิพัฒนา</t>
+          <t>แยกใต้ทางด่วนพระราม 9 (แยก RCA)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>หนองจอก</t>
+          <t>ห้วยขวาง</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -8639,27 +8629,27 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ความกว้างถนนไม่เพียงพอให้ปรับช่องจราจร</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ข้อจำกัดทางกายภาพ</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>13.8557481105835</v>
+        <v>13.7527203</v>
       </c>
       <c r="J19" t="n">
-        <v>100.853164957125</v>
+        <v>100.5743538</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>กรุงเทพตะวันออก</t>
+          <t>กรุงเทพกลาง</t>
         </is>
       </c>
     </row>
@@ -8669,17 +8659,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>จุดกลับรถหน้าหมู่บ้านศรีประจักษ์ ถนนรามคำแหง</t>
+          <t>แยกหทัยราษฎร์ตัดถนนสุเหร่าคลองหนึ่ง (แยกคอกม้า)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>สะพานสูง</t>
+          <t>คลองสามวา</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -8688,11 +8678,11 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร (แนวรถไฟฟ้าสายสีส้ม)</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -8701,10 +8691,10 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>13.787472</v>
+        <v>13.84173</v>
       </c>
       <c r="J20" t="n">
-        <v>100.6927</v>
+        <v>100.720501</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -8723,12 +8713,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>จุดกลับรถหน้าหมู่บ้านสัมมากร ประตู 2 ถนนรามคำแหง</t>
+          <t>คอขวดถนนเพิ่มสิน (บริเวณศาลเจ้าพ่อสมบุญ)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>สะพานสูง</t>
+          <t>สายไหม</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -8737,11 +8727,11 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ประชุมร่วม รฟม. เร่งคืนผิวจราจร (แนวรถไฟฟ้าสายสีส้ม)</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -8750,14 +8740,14 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>13.777225</v>
+        <v>13.903434</v>
       </c>
       <c r="J21" t="n">
-        <v>100.674031</v>
+        <v>100.622861</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>กรุงเทพตะวันออก</t>
+          <t>กรุงเทพเหนือ</t>
         </is>
       </c>
     </row>
@@ -8767,17 +8757,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2567/2568</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>แยกคลองเจ็ก ถนนรามคำแหง</t>
+          <t>จุดกลับรถถนนเพชรเกษม (บริเวณซอยเพชรเกษม 116 และซอยเพชรเกษม 81/4)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>สะพานสูง</t>
+          <t>หนองแขม</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -8786,7 +8776,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>62.5</v>
+        <v>25</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -8799,14 +8789,14 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>13.78197222</v>
+        <v>13.705046</v>
       </c>
       <c r="J22" t="n">
-        <v>100.6828333</v>
+        <v>100.337723</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>กรุงเทพตะวันออก</t>
+          <t>กรุงธนใต้</t>
         </is>
       </c>
     </row>
@@ -8821,12 +8811,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>แยกหทัยราษฎร์ตัดถนนสุเหร่าคลองหนึ่ง (แยกคอกม้า)</t>
+          <t>แยกหน้าทางเข้าโรงเรียนปาณยาพัฒนาการ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>คลองสามวา</t>
+          <t>สวนหลวง</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -8835,7 +8825,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -8848,14 +8838,14 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>13.84173</v>
+        <v>13.737036</v>
       </c>
       <c r="J23" t="n">
-        <v>100.720501</v>
+        <v>100.626139</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>กรุงเทพตะวันออก</t>
+          <t>กรุงเทพใต้</t>
         </is>
       </c>
     </row>
@@ -8870,12 +8860,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>คอขวดถนนเพิ่มสิน (บริเวณศาลเจ้าพ่อสมบุญ)</t>
+          <t>แยกคลองเจ็ก ถนนรามคำแหง</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>สายไหม</t>
+          <t>สะพานสูง</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -8884,7 +8874,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -8897,14 +8887,14 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>13.903434</v>
+        <v>13.78197222</v>
       </c>
       <c r="J24" t="n">
-        <v>100.622861</v>
+        <v>100.6828333</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>กรุงเทพเหนือ</t>
+          <t>กรุงเทพตะวันออก</t>
         </is>
       </c>
     </row>
@@ -8919,12 +8909,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>จุดกลับรถถนนเพชรเกษม (บริเวณซอยเพชรเกษม 116 และซอยเพชรเกษม 81/4)</t>
+          <t>แยกลาซาลตัดแบริ่ง</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>หนองแขม</t>
+          <t>บางนา</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -8933,7 +8923,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>25</v>
+        <v>81.25</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -8946,14 +8936,14 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>13.705046</v>
+        <v>13.660765</v>
       </c>
       <c r="J25" t="n">
-        <v>100.337723</v>
+        <v>100.624963</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>กรุงธนใต้</t>
+          <t>กรุงเทพใต้</t>
         </is>
       </c>
     </row>
@@ -8963,46 +8953,46 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2567</t>
+          <t>2568</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>แยกต่างระดับราชพฤกษ์ - รัชดาภิเษก</t>
+          <t>แยกศรีนครินทร์-ลาซาล (แยกศรีลาซาล)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ธนบุรี</t>
+          <t>บางนา</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ทช.</t>
+          <t>กทม.</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>81.25</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>อยู่ในความรับผิดชอบ ทช. (กรมทางหลวงชนบท)</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>นอกอำนาจ กทม.</t>
+          <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>13.7154111</v>
+        <v>13.65622</v>
       </c>
       <c r="J26" t="n">
-        <v>100.4782633</v>
+        <v>100.642369</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>กรุงธนเหนือ</t>
+          <t>กรุงเทพใต้</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill remarks for Sriprajak & Sammakorn U-turn points: 'in progress' (user-confirmed); blank remark + 1-99% now defaults to in-progress in rebuild script
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8548,6 +8548,11 @@
           <t>อยู่ระหว่างดำเนินการ</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>อยู่ระหว่างดำเนินการ</t>
+        </is>
+      </c>
       <c r="I17" t="n">
         <v>13.787472</v>
       </c>
@@ -8588,6 +8593,11 @@
         <v>5</v>
       </c>
       <c r="G18" t="inlineStr">
+        <is>
+          <t>อยู่ระหว่างดำเนินการ</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>อยู่ระหว่างดำเนินการ</t>
         </is>

</xml_diff>